<commit_message>
이슈 수집: 2026-06-24 06:11
</commit_message>
<xml_diff>
--- a/meki_이슈_히스토리.xlsx
+++ b/meki_이슈_히스토리.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +37,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +57,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C8A870"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,13 +91,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,7 +470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -523,6 +538,35 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="52" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>아레나 콜로세움 미적용</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>아레나 콜로세움 미적용</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr"/>
+      <c r="G3" s="4" t="inlineStr"/>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
이슈 수집: 2026-06-24 06:13
</commit_message>
<xml_diff>
--- a/meki_이슈_히스토리.xlsx
+++ b/meki_이슈_히스토리.xlsx
@@ -42,7 +42,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9F9F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -103,6 +108,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -470,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -567,6 +578,35 @@
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="4" t="inlineStr"/>
     </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>아레나 수치 적용</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>아레나 수치 적용</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr"/>
+      <c r="G4" s="6" t="inlineStr"/>
+      <c r="H4" s="5" t="inlineStr"/>
+      <c r="I4" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>